<commit_message>
Save generated outputs and update viewer (undo/redo + header editing)
</commit_message>
<xml_diff>
--- a/timetable_generator/timetable_outputs/CSE_Sem1_SectionA_Timetable.xlsx
+++ b/timetable_generator/timetable_outputs/CSE_Sem1_SectionA_Timetable.xlsx
@@ -485,18 +485,18 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CS161
+Problem solving through programming 
+C101
+Dr. Sunil P V</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>EC161
-Digital Design 
-C101
-Dr. Prakash Pawar</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -504,18 +504,19 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EC161
+Digital Design 
+C101
+Dr. Prakash Pawar
+[COMMON]</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>EC161
-Digital Design 
-C101
-Dr. Prakash Pawar</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -523,17 +524,27 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>EC161
 Digital Design 
 C101
-Dr. Prakash Pawar</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+Dr. Prakash Pawar
+[COMMON]</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EC161
+Digital Design 
+C101
+Dr. Prakash Pawar
+[COMMON]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>CS161
 Problem solving through programming 
@@ -541,7 +552,6 @@
 Dr. Sunil P V</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -567,14 +577,7 @@
 Dr. Sunil P V</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CS161
-Problem solving through programming 
-C101
-Dr. Sunil P V</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>